<commit_message>
PRO v2: hoja Monedas (conversor tasa del dia) + moneda en lista
</commit_message>
<xml_diff>
--- a/CalculadoraPRO.xlsx
+++ b/CalculadoraPRO.xlsx
@@ -9,7 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calculadora" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A cuanto vendo" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Como usarla" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monedas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Como usarla" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,42 +30,59 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="007B2FF7"/>
-      <sz val="14"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
     </font>
     <font>
       <i val="1"/>
-      <color rgb="00666666"/>
+      <color rgb="008B7BA8"/>
       <sz val="9"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="12"/>
+      <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="002F6B4F"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001B5E20"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001B5E20"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001B5E20"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001B5E20"/>
+      <sz val="16"/>
     </font>
     <font>
       <b val="1"/>
     </font>
     <font>
-      <b val="1"/>
-      <color rgb="002F6B4F"/>
-      <sz val="13"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="002F6B4F"/>
-      <sz val="16"/>
+      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -73,12 +91,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="005B1E9E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5EDFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="007B2FF7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A8FF78"/>
+        <fgColor rgb="00E8F5E9"/>
       </patternFill>
     </fill>
   </fills>
@@ -94,18 +122,34 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -468,18 +512,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="007B2FF7"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -492,256 +537,335 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Columnas B, C y D se escriben. E y F se calculan solas.</t>
+          <t>Todo se calcula SOLO. Tú escribes B, C y D. La ganancia real ya trae la comisión descontada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Moneda de la lista:</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>CUP</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>← elige: CUP, USD, EUR, MLC, CAD (vale para cualquier moneda)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Producto</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>¿Cuánto te costó?</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Costo</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Precio de venta</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>Comisión % (transferencia)</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>GANANCIA REAL</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>Margen %</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Café (libra)</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="7" t="n">
         <v>800</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="7" t="n">
         <v>1200</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="8">
         <f>IF(OR(B5="",C5=""),"",C5*(1-D5/100)-B5)</f>
         <v/>
       </c>
-      <c r="F5">
+      <c r="F5" s="8">
         <f>IF(OR(B5="",C5="",C5=0),"",(C5*(1-D5/100)-B5)/C5*100)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Cigarro (caja)</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="7" t="n">
         <v>2500</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" s="7" t="n">
         <v>3500</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6" s="8">
         <f>IF(OR(B6="",C6=""),"",C6*(1-D6/100)-B6)</f>
         <v/>
       </c>
-      <c r="F6">
+      <c r="F6" s="8">
         <f>IF(OR(B6="",C6="",C6=0),"",(C6*(1-D6/100)-B6)/C6*100)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Pan (unidad)</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="7" t="n">
         <v>60</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7" s="7" t="n">
         <v>120</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E7" s="8">
         <f>IF(OR(B7="",C7=""),"",C7*(1-D7/100)-B7)</f>
         <v/>
       </c>
-      <c r="F7">
+      <c r="F7" s="8">
         <f>IF(OR(B7="",C7="",C7=0),"",(C7*(1-D7/100)-B7)/C7*100)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="E8" s="4">
+      <c r="A8" s="6" t="n"/>
+      <c r="B8" s="7" t="n"/>
+      <c r="C8" s="7" t="n"/>
+      <c r="D8" s="7" t="n"/>
+      <c r="E8" s="8">
         <f>IF(OR(B8="",C8=""),"",C8*(1-D8/100)-B8)</f>
         <v/>
       </c>
-      <c r="F8">
+      <c r="F8" s="8">
         <f>IF(OR(B8="",C8="",C8=0),"",(C8*(1-D8/100)-B8)/C8*100)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="E9" s="4">
+      <c r="A9" s="6" t="n"/>
+      <c r="B9" s="7" t="n"/>
+      <c r="C9" s="7" t="n"/>
+      <c r="D9" s="7" t="n"/>
+      <c r="E9" s="8">
         <f>IF(OR(B9="",C9=""),"",C9*(1-D9/100)-B9)</f>
         <v/>
       </c>
-      <c r="F9">
+      <c r="F9" s="8">
         <f>IF(OR(B9="",C9="",C9=0),"",(C9*(1-D9/100)-B9)/C9*100)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="E10" s="4">
+      <c r="A10" s="6" t="n"/>
+      <c r="B10" s="7" t="n"/>
+      <c r="C10" s="7" t="n"/>
+      <c r="D10" s="7" t="n"/>
+      <c r="E10" s="8">
         <f>IF(OR(B10="",C10=""),"",C10*(1-D10/100)-B10)</f>
         <v/>
       </c>
-      <c r="F10">
+      <c r="F10" s="8">
         <f>IF(OR(B10="",C10="",C10=0),"",(C10*(1-D10/100)-B10)/C10*100)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="E11" s="4">
+      <c r="A11" s="6" t="n"/>
+      <c r="B11" s="7" t="n"/>
+      <c r="C11" s="7" t="n"/>
+      <c r="D11" s="7" t="n"/>
+      <c r="E11" s="8">
         <f>IF(OR(B11="",C11=""),"",C11*(1-D11/100)-B11)</f>
         <v/>
       </c>
-      <c r="F11">
+      <c r="F11" s="8">
         <f>IF(OR(B11="",C11="",C11=0),"",(C11*(1-D11/100)-B11)/C11*100)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="E12" s="4">
+      <c r="A12" s="6" t="n"/>
+      <c r="B12" s="7" t="n"/>
+      <c r="C12" s="7" t="n"/>
+      <c r="D12" s="7" t="n"/>
+      <c r="E12" s="8">
         <f>IF(OR(B12="",C12=""),"",C12*(1-D12/100)-B12)</f>
         <v/>
       </c>
-      <c r="F12">
+      <c r="F12" s="8">
         <f>IF(OR(B12="",C12="",C12=0),"",(C12*(1-D12/100)-B12)/C12*100)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="E13" s="4">
+      <c r="A13" s="6" t="n"/>
+      <c r="B13" s="7" t="n"/>
+      <c r="C13" s="7" t="n"/>
+      <c r="D13" s="7" t="n"/>
+      <c r="E13" s="8">
         <f>IF(OR(B13="",C13=""),"",C13*(1-D13/100)-B13)</f>
         <v/>
       </c>
-      <c r="F13">
+      <c r="F13" s="8">
         <f>IF(OR(B13="",C13="",C13=0),"",(C13*(1-D13/100)-B13)/C13*100)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="E14" s="4">
+      <c r="A14" s="6" t="n"/>
+      <c r="B14" s="7" t="n"/>
+      <c r="C14" s="7" t="n"/>
+      <c r="D14" s="7" t="n"/>
+      <c r="E14" s="8">
         <f>IF(OR(B14="",C14=""),"",C14*(1-D14/100)-B14)</f>
         <v/>
       </c>
-      <c r="F14">
+      <c r="F14" s="8">
         <f>IF(OR(B14="",C14="",C14=0),"",(C14*(1-D14/100)-B14)/C14*100)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="E15" s="4">
+      <c r="A15" s="6" t="n"/>
+      <c r="B15" s="7" t="n"/>
+      <c r="C15" s="7" t="n"/>
+      <c r="D15" s="7" t="n"/>
+      <c r="E15" s="8">
         <f>IF(OR(B15="",C15=""),"",C15*(1-D15/100)-B15)</f>
         <v/>
       </c>
-      <c r="F15">
+      <c r="F15" s="8">
         <f>IF(OR(B15="",C15="",C15=0),"",(C15*(1-D15/100)-B15)/C15*100)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="E16" s="4">
+      <c r="A16" s="6" t="n"/>
+      <c r="B16" s="7" t="n"/>
+      <c r="C16" s="7" t="n"/>
+      <c r="D16" s="7" t="n"/>
+      <c r="E16" s="8">
         <f>IF(OR(B16="",C16=""),"",C16*(1-D16/100)-B16)</f>
         <v/>
       </c>
-      <c r="F16">
+      <c r="F16" s="8">
         <f>IF(OR(B16="",C16="",C16=0),"",(C16*(1-D16/100)-B16)/C16*100)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="E17" s="4">
+      <c r="A17" s="6" t="n"/>
+      <c r="B17" s="7" t="n"/>
+      <c r="C17" s="7" t="n"/>
+      <c r="D17" s="7" t="n"/>
+      <c r="E17" s="8">
         <f>IF(OR(B17="",C17=""),"",C17*(1-D17/100)-B17)</f>
         <v/>
       </c>
-      <c r="F17">
+      <c r="F17" s="8">
         <f>IF(OR(B17="",C17="",C17=0),"",(C17*(1-D17/100)-B17)/C17*100)</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="E18" s="4">
+      <c r="A18" s="6" t="n"/>
+      <c r="B18" s="7" t="n"/>
+      <c r="C18" s="7" t="n"/>
+      <c r="D18" s="7" t="n"/>
+      <c r="E18" s="8">
         <f>IF(OR(B18="",C18=""),"",C18*(1-D18/100)-B18)</f>
         <v/>
       </c>
-      <c r="F18">
+      <c r="F18" s="8">
         <f>IF(OR(B18="",C18="",C18=0),"",(C18*(1-D18/100)-B18)/C18*100)</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="E19" s="4">
+      <c r="A19" s="6" t="n"/>
+      <c r="B19" s="7" t="n"/>
+      <c r="C19" s="7" t="n"/>
+      <c r="D19" s="7" t="n"/>
+      <c r="E19" s="8">
         <f>IF(OR(B19="",C19=""),"",C19*(1-D19/100)-B19)</f>
         <v/>
       </c>
-      <c r="F19">
+      <c r="F19" s="8">
         <f>IF(OR(B19="",C19="",C19=0),"",(C19*(1-D19/100)-B19)/C19*100)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="E20" s="4">
+      <c r="A20" s="6" t="n"/>
+      <c r="B20" s="7" t="n"/>
+      <c r="C20" s="7" t="n"/>
+      <c r="D20" s="7" t="n"/>
+      <c r="E20" s="8">
         <f>IF(OR(B20="",C20=""),"",C20*(1-D20/100)-B20)</f>
         <v/>
       </c>
-      <c r="F20">
+      <c r="F20" s="8">
         <f>IF(OR(B20="",C20="",C20=0),"",(C20*(1-D20/100)-B20)/C20*100)</f>
         <v/>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>GANANCIA TOTAL de la lista:</t>
-        </is>
-      </c>
-      <c r="E23" s="6">
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>GANANCIA TOTAL de la lista (en tu moneda):</t>
+        </is>
+      </c>
+      <c r="E21" s="10">
         <f>SUM(E5:E20)</f>
         <v/>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="C3:F3"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="B3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"CUP,USD,EUR,MLC,CAD"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -749,72 +873,94 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00F72FB8"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🎯 ¿Quieres ganar X? Aquí te digo a cuánto vender (comisión incluida)</t>
-        </is>
+          <t>🎯 ¿Quieres ganar X? Aquí te digo a cuánto vender</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>¿Cuánto te costó?</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="n">
+        <v>800</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>¿Cuánto te costó?</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>800</v>
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>¿Cuánto quieres ganar?</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="n">
+        <v>300</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>¿Cuánto quieres ganar?</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>300</v>
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Comisión % (transferencia)</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Comisión % (transferencia)</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>2</v>
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>PONLE ESTE PRECIO:</t>
+        </is>
+      </c>
+      <c r="B5" s="12">
+        <f>(B2+B3)/(1-B4/100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>(comisión ya incluida — redondea hacia arriba y nadie se molesta 😉)</t>
+        </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>PONLE ESTE PRECIO:</t>
-        </is>
-      </c>
-      <c r="B7" s="8">
-        <f>(B3+B4)/(1-B5/100)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>(redondea hacia arriba y nadie se molesta 😉)</t>
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Moneda (para tu referencia):</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>CUP</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="B7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"CUP,USD,EUR,MLC,CAD"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -822,86 +968,269 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="0000C853"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="75" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>💱 CONVERSOR DE MONEDAS — funciona en cualquier moneda</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Pon la TASA DEL DÍA en la columna blanca (cambian a diario). Las de abajo son solo ejemplo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>Moneda</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>Cuánto vale en CUP (tasa del día)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>CUP</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>MLC</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>CAD</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>Cantidad a convertir:</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>De la moneda:</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>A la moneda:</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>CUP</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>RECIBES:</t>
+        </is>
+      </c>
+      <c r="B14" s="12">
+        <f>IF(OR(B11="",B12="",B13=""),"",B11*VLOOKUP(B12,$A$5:$B$9,2,0)/VLOOKUP(B13,$A$5:$B$9,2,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>💡 Compraste en USD y vendes en CUP (o EUR, MLC...)? Convierte tu costo aquí y ponlo en la hoja 'Calculadora'.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="B12 B13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=$A$5:$A$9</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00FFC107"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="95" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
           <t>📘 CÓMO USAR TU CALCULADORA PRO</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>1. TODO SE CALCULA SOLO: tú solo escribes en las casillas blancas. Nada de fórmulas.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>1. Hoja 'Calculadora': escribe producto, costo, precio y la comisión de la</t>
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>2. Hoja 'Calculadora': elige tu MONEDA arriba (CUP, USD, EUR, MLC, CAD). Escribe producto,</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   transferencia (en Cuba suele ser 2-4%, pon la tuya). La GANANCIA REAL y el</t>
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   costo, precio y la comisión % de la transferencia (en Cuba suele ser 2-4%).</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   margen se calculan solos — ya con la comisión descontada.</t>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   La GANANCIA REAL y el margen salen solos — ya con la comisión descontada.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2. Hoja 'A cuanto vendo': pon cuánto te costó y cuánto QUIERES ganar, y te</t>
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>3. Hoja 'A cuanto vendo': pon cuánto te costó y cuánto quieres ganar → te da el precio</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   dice el precio exacto (comisión incluida, para que no pierdas ni un peso).</t>
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   exacto para ponerle (comisión incluida).</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>3. Las casillas con ejemplos (café, cigarro, pan) se borran y escribes las tuyas.</t>
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>4. Hoja 'Monedas': pon las tasas del día y convierte cualquier cantidad entre monedas</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>4. Funciona SIN internet en Excel, WPS o Google Sheets. Guárdala en el teléfono.</t>
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   (USD, EUR, MLC, CUP, CAD...). Ideal si compras en una moneda y vendes en otra.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>5. Las casillas con ejemplos (café, cigarro, pan, tasas 400/250/300) son solo ejemplos:</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   escríbeles encima con tus números.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>6. Funciona SIN internet en Excel, WPS Office o Google Sheets. Es tuya para siempre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>🚀 Hecho por DESPEGUE DIGITAL — t.me/Despeguedijitalbot</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="16" t="inlineStr">
         <is>
           <t>🛒 Más herramientas para tu negocio: https://mia9911.github.io/despegue-digital/</t>
         </is>

</xml_diff>